<commit_message>
Evento #2 registrado en reporte_2026-06-24.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-24.xlsx
+++ b/datos/excel/reporte_2026-06-24.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,51 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>🚨 SÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>07:03:10</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>273.44</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-16.79</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>562.5 Hz | 789.1 Hz | 1140.6 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2888</v>
+      </c>
+      <c r="J3" t="n">
+        <v>130</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evento #3 registrado en reporte_2026-06-24.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-24.xlsx
+++ b/datos/excel/reporte_2026-06-24.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,51 @@
         <v>130</v>
       </c>
       <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>07:03:26</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>695.3099999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-25.73</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1343.8 Hz | 2125.0 Hz | 2796.9 Hz</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2517</v>
+      </c>
+      <c r="J4" t="n">
+        <v>58</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #4 registrado en reporte_2026-06-24.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-24.xlsx
+++ b/datos/excel/reporte_2026-06-24.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,51 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>07:03:39</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>382.81</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-28.26</v>
+      </c>
+      <c r="G5" t="n">
+        <v>70</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>765.6 Hz | 1171.9 Hz | 1554.7 Hz</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>2554</v>
+      </c>
+      <c r="J5" t="n">
+        <v>59</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evento #5 registrado en reporte_2026-06-24.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-24.xlsx
+++ b/datos/excel/reporte_2026-06-24.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -650,6 +650,51 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>🚨 SÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>07:03:50</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>304.69</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-29.52</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>648.4 Hz | 898.4 Hz | 1203.1 Hz</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>2533</v>
+      </c>
+      <c r="J6" t="n">
+        <v>59</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evento #6 registrado en reporte_2026-06-24.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-24.xlsx
+++ b/datos/excel/reporte_2026-06-24.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,6 +695,51 @@
       <c r="K6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>07:04:00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>500</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-29.29</v>
+      </c>
+      <c r="G7" t="n">
+        <v>70</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1007.8 Hz | 1523.4 Hz | 1960.9 Hz</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>2519</v>
+      </c>
+      <c r="J7" t="n">
+        <v>57</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>